<commit_message>
Update test case generation script with improved summary sheet and additional test cases
Adjusted column header casing in `scripts/generate-test-cases.cjs` and updated the `PMS_Test_Cases_Comprehensive.xlsx` file to include more test scenarios and refine the summary sheet's formulas.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 3a47d2e3-af4e-4b6d-b1c5-2ab503fcf377
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: bdcc4a3d-bd70-4079-834f-9bcc1a363306
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/PMS_Test_Cases_Comprehensive.xlsx
+++ b/PMS_Test_Cases_Comprehensive.xlsx
@@ -170,40 +170,40 @@
     <t>(To be updated during testing)</t>
   </si>
   <si>
-    <t>TEST CASE ID</t>
-  </si>
-  <si>
-    <t>MODULE/SECTION</t>
-  </si>
-  <si>
-    <t>TEST SCENARIO</t>
-  </si>
-  <si>
-    <t>PRIORITY</t>
-  </si>
-  <si>
-    <t>TEST STEPS</t>
-  </si>
-  <si>
-    <t>TEST DATA</t>
-  </si>
-  <si>
-    <t>EXPECTED RESULT</t>
-  </si>
-  <si>
-    <t>ACTUAL RESULT</t>
-  </si>
-  <si>
-    <t>PASS/FAIL</t>
-  </si>
-  <si>
-    <t>COMMENTS/ISSUES</t>
-  </si>
-  <si>
-    <t>TESTER NAME</t>
-  </si>
-  <si>
-    <t>TEST DATE</t>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>Module/Section</t>
+  </si>
+  <si>
+    <t>Test Scenario</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Test Steps</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Pass/Fail</t>
+  </si>
+  <si>
+    <t>Comments/Issues</t>
+  </si>
+  <si>
+    <t>Tester Name</t>
+  </si>
+  <si>
+    <t>Test Date</t>
   </si>
   <si>
     <t>COMP-001</t>

</xml_diff>